<commit_message>
feat: add iam group column support for folder creation in data wizard
</commit_message>
<xml_diff>
--- a/backend/data_wizard/tests/templates/sample_folders.xlsx
+++ b/backend/data_wizard/tests/templates/sample_folders.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -32,12 +32,18 @@
     <t xml:space="preserve">domain</t>
   </si>
   <si>
+    <t xml:space="preserve">iam_group</t>
+  </si>
+  <si>
     <t xml:space="preserve">ACME Corp</t>
   </si>
   <si>
     <t xml:space="preserve">Root domain for ACME</t>
   </si>
   <si>
+    <t xml:space="preserve">x</t>
+  </si>
+  <si>
     <t xml:space="preserve">IT Department</t>
   </si>
   <si>
@@ -78,6 +84,9 @@
   </si>
   <si>
     <t xml:space="preserve">Name of the parent folder. Leave blank to place the folder at root level. Must match exactly one existing folder name (case-insensitive). An error is returned when the name is ambiguous.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When non-empty (e.g. 'x'), enables IAM group creation for the folder (create_iam_groups).</t>
   </si>
 </sst>
 </file>
@@ -194,13 +203,21 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -467,65 +484,74 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3"/>
+      <c r="B2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>3</v>
+      <c r="A4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>3</v>
+      <c r="A5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -544,56 +570,67 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="90"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>15</v>
+      <c r="B2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>17</v>
+      <c r="B3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>18</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>